<commit_message>
23.09.2026 pred kraj dana
</commit_message>
<xml_diff>
--- a/testdata/configuration.xlsx
+++ b/testdata/configuration.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="63">
   <si>
     <t>Order</t>
   </si>
@@ -143,7 +143,7 @@
     <t>dev</t>
   </si>
   <si>
-    <t>https://test.dbp.nlbkb.rs/login</t>
+    <t>https://uat.dbp.nlbkb.rs/login</t>
   </si>
   <si>
     <t>Chrome</t>
@@ -161,16 +161,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>rs.nlb.klik.tst:id/</t>
-  </si>
-  <si>
-    <t>rs.nlb.klik.test</t>
+    <t>rs.nlb.klik.uat:id/</t>
+  </si>
+  <si>
+    <t>rs.nlb.klik.uat</t>
   </si>
   <si>
     <t>si.nlb.klik.RootActivity</t>
-  </si>
-  <si>
-    <t>si.nlb.klik.uat:id/</t>
   </si>
   <si>
     <t>emulator-5554</t>
@@ -1334,6 +1331,7 @@
     <col min="8" max="9" width="22.5740740740741" customWidth="1"/>
     <col min="10" max="12" width="31.712962962963" customWidth="1"/>
     <col min="13" max="13" width="16.4259259259259" customWidth="1"/>
+    <col min="14" max="14" width="22.5555555555556" customWidth="1"/>
     <col min="20" max="20" width="16.4259259259259" customWidth="1"/>
     <col min="21" max="21" width="12.287037037037" customWidth="1"/>
     <col min="31" max="31" width="16" customWidth="1"/>
@@ -1488,88 +1486,88 @@
         <v>46</v>
       </c>
       <c r="L2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="V2" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="V2" s="8" t="s">
+      <c r="W2" t="s">
+        <v>52</v>
+      </c>
+      <c r="X2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE2" t="s">
         <v>57</v>
       </c>
-      <c r="W2" t="s">
-        <v>53</v>
-      </c>
-      <c r="X2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE2" t="s">
+      <c r="AF2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="AF2" s="9" t="s">
+      <c r="AG2" t="s">
         <v>59</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>60</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="AI2" s="9" t="s">
-        <v>62</v>
       </c>
       <c r="AJ2" s="5" t="s">
         <v>41</v>
       </c>
       <c r="AK2" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="AF2" r:id="rId1" display="bozidar.tomasevic@dtc.rs"/>
-    <hyperlink ref="C2" r:id="rId2" display="https://test.dbp.nlbkb.rs/login" tooltip="https://test.dbp.nlbkb.rs/login"/>
+    <hyperlink ref="C2" r:id="rId2" display="https://uat.dbp.nlbkb.rs/login" tooltip="https://uat.dbp.nlbkb.rs/login"/>
     <hyperlink ref="AI2" r:id="rId3" display="\\10.11.1.158\03. TEST Team\NLB SLO\FileShare\UAT" tooltip="\\10.11.1.158\03. TEST Team\NLB SLO\FileShare\UAT"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>